<commit_message>
Add IPL cricket project
</commit_message>
<xml_diff>
--- a/Reports/Data_Dictionary_Template.xlsx
+++ b/Reports/Data_Dictionary_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muham\Works\project 3.1\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48CC71AA-3FA8-493E-8729-B4EED40C0570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4DC0012-5A9D-4F2D-86B1-43E0B6A9C43D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -174,9 +174,6 @@
     <t>Trainee name</t>
   </si>
   <si>
-    <t>[Your name]</t>
-  </si>
-  <si>
     <t>Date prepared</t>
   </si>
   <si>
@@ -607,6 +604,9 @@
   </si>
   <si>
     <t>Handle when converting season to year</t>
+  </si>
+  <si>
+    <t>Muhammad Sinan PS</t>
   </si>
 </sst>
 </file>
@@ -871,19 +871,19 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1358,55 +1358,55 @@
         <v>40</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>41</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="12" t="s">
         <v>44</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>46</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>50</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>52</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1429,88 +1429,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
-      <c r="S2" s="31"/>
-      <c r="T2" s="31"/>
-      <c r="U2" s="31"/>
+      <c r="A2" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="32"/>
+      <c r="T2" s="32"/>
+      <c r="U2" s="32"/>
     </row>
     <row r="4" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
-      <c r="O4" s="32"/>
-      <c r="P4" s="32"/>
-      <c r="Q4" s="32"/>
-      <c r="R4" s="32"/>
-      <c r="S4" s="32"/>
-      <c r="T4" s="32"/>
-      <c r="U4" s="32"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="34"/>
+      <c r="K4" s="34"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="34"/>
+      <c r="O4" s="34"/>
+      <c r="P4" s="34"/>
+      <c r="Q4" s="34"/>
+      <c r="R4" s="34"/>
+      <c r="S4" s="34"/>
+      <c r="T4" s="34"/>
+      <c r="U4" s="34"/>
     </row>
     <row r="5" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="33" t="s">
         <v>57</v>
-      </c>
-      <c r="B5" s="33" t="s">
-        <v>58</v>
       </c>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
@@ -1534,45 +1534,45 @@
     </row>
     <row r="6" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="34" t="s">
-        <v>62</v>
-      </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="34"/>
-      <c r="Q6" s="34"/>
-      <c r="R6" s="34"/>
-      <c r="S6" s="34"/>
-      <c r="T6" s="34"/>
-      <c r="U6" s="34"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="35"/>
+      <c r="O6" s="35"/>
+      <c r="P6" s="35"/>
+      <c r="Q6" s="35"/>
+      <c r="R6" s="35"/>
+      <c r="S6" s="35"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="35"/>
     </row>
     <row r="7" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13"/>
       <c r="B7" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="33" t="s">
         <v>64</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>65</v>
       </c>
       <c r="E7" s="33"/>
       <c r="F7" s="33"/>
@@ -1594,37 +1594,37 @@
     </row>
     <row r="8" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="32"/>
-      <c r="N8" s="32"/>
-      <c r="O8" s="32"/>
-      <c r="P8" s="32"/>
-      <c r="Q8" s="32"/>
-      <c r="R8" s="32"/>
-      <c r="S8" s="32"/>
-      <c r="T8" s="32"/>
-      <c r="U8" s="32"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="34"/>
+      <c r="M8" s="34"/>
+      <c r="N8" s="34"/>
+      <c r="O8" s="34"/>
+      <c r="P8" s="34"/>
+      <c r="Q8" s="34"/>
+      <c r="R8" s="34"/>
+      <c r="S8" s="34"/>
+      <c r="T8" s="34"/>
+      <c r="U8" s="34"/>
     </row>
     <row r="9" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B9" s="33" t="s">
         <v>68</v>
-      </c>
-      <c r="B9" s="33" t="s">
-        <v>69</v>
       </c>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
@@ -1648,13 +1648,13 @@
     </row>
     <row r="10" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
@@ -1705,25 +1705,25 @@
     <row r="12" spans="1:21" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:21" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="C13" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="D13" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="E13" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="F13" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="G13" s="20" t="s">
         <v>78</v>
-      </c>
-      <c r="G13" s="20" t="s">
-        <v>79</v>
       </c>
       <c r="H13" s="20"/>
       <c r="I13" s="20"/>
@@ -1742,25 +1742,25 @@
     </row>
     <row r="14" spans="1:21" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="C14" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="D14" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="E14" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="F14" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="G14" s="21" t="s">
         <v>85</v>
-      </c>
-      <c r="G14" s="21" t="s">
-        <v>86</v>
       </c>
       <c r="H14" s="21"/>
       <c r="I14" s="21"/>
@@ -1779,25 +1779,25 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B15" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="C15" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="D15" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="E15" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="F15" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H15" s="21"/>
       <c r="I15" s="21"/>
@@ -1816,25 +1816,25 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="C16" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="D16" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="G16" s="21" t="s">
         <v>94</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="F16" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="G16" s="21" t="s">
-        <v>95</v>
       </c>
       <c r="H16" s="21"/>
       <c r="I16" s="21"/>
@@ -1853,25 +1853,25 @@
     </row>
     <row r="17" spans="1:21" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="21" t="s">
+      <c r="C17" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="D17" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="E17" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="F17" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="G17" s="21" t="s">
         <v>101</v>
-      </c>
-      <c r="G17" s="21" t="s">
-        <v>102</v>
       </c>
       <c r="H17" s="21"/>
       <c r="I17" s="21"/>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B18" s="23">
         <v>50000</v>
@@ -1902,7 +1902,7 @@
         <v>8</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F18" s="23">
         <v>3</v>
@@ -1927,25 +1927,25 @@
     </row>
     <row r="19" spans="1:21" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="B19" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="D19" s="21" t="s">
+      <c r="E19" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="F19" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="E19" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="F19" s="21" t="s">
-        <v>107</v>
-      </c>
       <c r="G19" s="21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H19" s="21"/>
       <c r="I19" s="21"/>
@@ -1964,25 +1964,25 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="C20" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C20" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="E20" s="21" t="s">
+      <c r="F20" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="G20" s="21" t="s">
         <v>110</v>
-      </c>
-      <c r="F20" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="G20" s="21" t="s">
-        <v>111</v>
       </c>
       <c r="H20" s="21"/>
       <c r="I20" s="21"/>
@@ -2001,25 +2001,25 @@
     </row>
     <row r="21" spans="1:21" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="C21" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="E21" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="C21" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="E21" s="21" t="s">
+      <c r="F21" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="G21" s="21" t="s">
         <v>114</v>
-      </c>
-      <c r="F21" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="G21" s="21" t="s">
-        <v>115</v>
       </c>
       <c r="H21" s="21"/>
       <c r="I21" s="21"/>
@@ -2041,37 +2041,37 @@
     <row r="25" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="32"/>
-      <c r="K26" s="32"/>
-      <c r="L26" s="32"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="32"/>
-      <c r="O26" s="32"/>
-      <c r="P26" s="32"/>
-      <c r="Q26" s="32"/>
-      <c r="R26" s="32"/>
-      <c r="S26" s="32"/>
-      <c r="T26" s="32"/>
-      <c r="U26" s="32"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="34"/>
+      <c r="L26" s="34"/>
+      <c r="M26" s="34"/>
+      <c r="N26" s="34"/>
+      <c r="O26" s="34"/>
+      <c r="P26" s="34"/>
+      <c r="Q26" s="34"/>
+      <c r="R26" s="34"/>
+      <c r="S26" s="34"/>
+      <c r="T26" s="34"/>
+      <c r="U26" s="34"/>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="33" t="s">
         <v>57</v>
-      </c>
-      <c r="B27" s="33" t="s">
-        <v>58</v>
       </c>
       <c r="C27" s="33"/>
       <c r="D27" s="33"/>
@@ -2095,45 +2095,45 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="D28" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="D28" s="34" t="s">
-        <v>62</v>
-      </c>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="34"/>
-      <c r="K28" s="34"/>
-      <c r="L28" s="34"/>
-      <c r="M28" s="34"/>
-      <c r="N28" s="34"/>
-      <c r="O28" s="34"/>
-      <c r="P28" s="34"/>
-      <c r="Q28" s="34"/>
-      <c r="R28" s="34"/>
-      <c r="S28" s="34"/>
-      <c r="T28" s="34"/>
-      <c r="U28" s="34"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="35"/>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
+      <c r="N28" s="35"/>
+      <c r="O28" s="35"/>
+      <c r="P28" s="35"/>
+      <c r="Q28" s="35"/>
+      <c r="R28" s="35"/>
+      <c r="S28" s="35"/>
+      <c r="T28" s="35"/>
+      <c r="U28" s="35"/>
     </row>
     <row r="29" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="13"/>
       <c r="B29" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="D29" s="33" t="s">
         <v>64</v>
-      </c>
-      <c r="D29" s="33" t="s">
-        <v>65</v>
       </c>
       <c r="E29" s="33"/>
       <c r="F29" s="33"/>
@@ -2155,37 +2155,37 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="B30" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="32"/>
-      <c r="K30" s="32"/>
-      <c r="L30" s="32"/>
-      <c r="M30" s="32"/>
-      <c r="N30" s="32"/>
-      <c r="O30" s="32"/>
-      <c r="P30" s="32"/>
-      <c r="Q30" s="32"/>
-      <c r="R30" s="32"/>
-      <c r="S30" s="32"/>
-      <c r="T30" s="32"/>
-      <c r="U30" s="32"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="34"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34"/>
+      <c r="K30" s="34"/>
+      <c r="L30" s="34"/>
+      <c r="M30" s="34"/>
+      <c r="N30" s="34"/>
+      <c r="O30" s="34"/>
+      <c r="P30" s="34"/>
+      <c r="Q30" s="34"/>
+      <c r="R30" s="34"/>
+      <c r="S30" s="34"/>
+      <c r="T30" s="34"/>
+      <c r="U30" s="34"/>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" s="33" t="s">
         <v>68</v>
-      </c>
-      <c r="B31" s="33" t="s">
-        <v>69</v>
       </c>
       <c r="C31" s="33"/>
       <c r="D31" s="33"/>
@@ -2209,13 +2209,13 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -2265,25 +2265,25 @@
     </row>
     <row r="35" spans="1:21" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A35" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="C35" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="20" t="s">
+      <c r="D35" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="E35" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="E35" s="20" t="s">
+      <c r="F35" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="F35" s="20" t="s">
+      <c r="G35" s="20" t="s">
         <v>78</v>
-      </c>
-      <c r="G35" s="20" t="s">
-        <v>79</v>
       </c>
       <c r="H35" s="20"/>
       <c r="I35" s="20"/>
@@ -2302,25 +2302,25 @@
     </row>
     <row r="36" spans="1:21" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A36" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="21" t="s">
+      <c r="C36" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="D36" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="E36" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="E36" s="21" t="s">
+      <c r="F36" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="F36" s="21" t="s">
+      <c r="G36" s="21" t="s">
         <v>85</v>
-      </c>
-      <c r="G36" s="21" t="s">
-        <v>86</v>
       </c>
       <c r="H36" s="21"/>
       <c r="I36" s="21"/>
@@ -2339,25 +2339,25 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A37" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="B37" s="21" t="s">
+      <c r="C37" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="C37" s="21" t="s">
+      <c r="D37" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="E37" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="E37" s="21" t="s">
-        <v>91</v>
-      </c>
       <c r="F37" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G37" s="21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H37" s="21"/>
       <c r="I37" s="21"/>
@@ -2376,25 +2376,25 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A38" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="C38" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="D38" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="F38" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="G38" s="21" t="s">
         <v>94</v>
-      </c>
-      <c r="D38" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="E38" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="F38" s="21" t="s">
-        <v>94</v>
-      </c>
-      <c r="G38" s="21" t="s">
-        <v>95</v>
       </c>
       <c r="H38" s="21"/>
       <c r="I38" s="21"/>
@@ -2413,25 +2413,25 @@
     </row>
     <row r="39" spans="1:21" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="21" t="s">
+      <c r="C39" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="C39" s="21" t="s">
+      <c r="D39" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="E39" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="E39" s="21" t="s">
+      <c r="F39" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="F39" s="21" t="s">
+      <c r="G39" s="21" t="s">
         <v>101</v>
-      </c>
-      <c r="G39" s="21" t="s">
-        <v>102</v>
       </c>
       <c r="H39" s="21"/>
       <c r="I39" s="21"/>
@@ -2450,7 +2450,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B40" s="23">
         <v>50000</v>
@@ -2462,7 +2462,7 @@
         <v>8</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F40" s="23">
         <v>3</v>
@@ -2487,25 +2487,25 @@
     </row>
     <row r="41" spans="1:21" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C41" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D41" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="B41" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C41" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="D41" s="21" t="s">
+      <c r="E41" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="F41" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="E41" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="F41" s="21" t="s">
-        <v>107</v>
-      </c>
       <c r="G41" s="21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H41" s="21"/>
       <c r="I41" s="21"/>
@@ -2524,25 +2524,25 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="B42" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B42" s="21" t="s">
+      <c r="C42" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="E42" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C42" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="D42" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="E42" s="21" t="s">
+      <c r="F42" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="G42" s="21" t="s">
         <v>110</v>
-      </c>
-      <c r="F42" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="G42" s="21" t="s">
-        <v>111</v>
       </c>
       <c r="H42" s="21"/>
       <c r="I42" s="21"/>
@@ -2561,25 +2561,25 @@
     </row>
     <row r="43" spans="1:21" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B43" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B43" s="21" t="s">
+      <c r="C43" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="E43" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="C43" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D43" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="E43" s="21" t="s">
+      <c r="F43" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="G43" s="21" t="s">
         <v>114</v>
-      </c>
-      <c r="F43" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="G43" s="21" t="s">
-        <v>115</v>
       </c>
       <c r="H43" s="21"/>
       <c r="I43" s="21"/>
@@ -2632,63 +2632,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
-        <v>116</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
+      <c r="A2" s="32" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
     </row>
     <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="B4" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="C4" s="25" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="D4" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="E4" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="F4" s="25" t="s">
         <v>121</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" s="21" t="s">
+      <c r="D5" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="D5" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E5" s="21" t="s">
+      <c r="F5" s="21" t="s">
         <v>125</v>
-      </c>
-      <c r="F5" s="21" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -2798,43 +2798,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
-        <v>127</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
+      <c r="A2" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
     </row>
     <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="C4" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="D4" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="E4" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="F4" s="25" t="s">
         <v>132</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2850,20 +2850,20 @@
         <f t="shared" ref="A6:A20" si="0">ROW()-5</f>
         <v>1</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="D6" s="30" t="s">
         <v>152</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="E6" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="E6" s="35" t="s">
-        <v>154</v>
-      </c>
-      <c r="F6" s="35" t="s">
-        <v>135</v>
+      <c r="F6" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -2871,20 +2871,20 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="D7" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="E7" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="D7" s="35" t="s">
-        <v>153</v>
-      </c>
-      <c r="E7" s="35" t="s">
-        <v>157</v>
-      </c>
-      <c r="F7" s="35" t="s">
-        <v>135</v>
+      <c r="F7" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -2892,20 +2892,20 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="C8" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="C8" s="35" t="s">
+      <c r="D8" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="D8" s="35" t="s">
+      <c r="E8" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="E8" s="35" t="s">
-        <v>161</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>135</v>
+      <c r="F8" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -2913,20 +2913,20 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B9" s="35" t="s">
-        <v>158</v>
-      </c>
-      <c r="C9" s="35" t="s">
+      <c r="B9" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="E9" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="D9" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="E9" s="35" t="s">
-        <v>163</v>
-      </c>
-      <c r="F9" s="35" t="s">
-        <v>135</v>
+      <c r="F9" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -2934,20 +2934,20 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="C10" s="35" t="s">
+      <c r="D10" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E10" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="D10" s="35" t="s">
-        <v>160</v>
-      </c>
-      <c r="E10" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="F10" s="35" t="s">
-        <v>135</v>
+      <c r="F10" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -2955,20 +2955,20 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B11" s="35" t="s">
-        <v>164</v>
-      </c>
-      <c r="C11" s="35" t="s">
+      <c r="B11" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E11" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="D11" s="35" t="s">
-        <v>160</v>
-      </c>
-      <c r="E11" s="35" t="s">
-        <v>168</v>
-      </c>
-      <c r="F11" s="35" t="s">
-        <v>135</v>
+      <c r="F11" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -2976,20 +2976,20 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="C12" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="C12" s="35" t="s">
-        <v>170</v>
-      </c>
-      <c r="D12" s="35" t="s">
+      <c r="D12" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="F12" s="30" t="s">
         <v>134</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -2997,20 +2997,20 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="C13" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="C13" s="35" t="s">
+      <c r="D13" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="E13" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="D13" s="35" t="s">
+      <c r="F13" s="30" t="s">
         <v>134</v>
-      </c>
-      <c r="E13" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="F13" s="35" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -3018,20 +3018,20 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="C14" s="30" t="s">
         <v>174</v>
       </c>
-      <c r="C14" s="35" t="s">
+      <c r="D14" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="E14" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="D14" s="35" t="s">
-        <v>153</v>
-      </c>
-      <c r="E14" s="35" t="s">
-        <v>176</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>135</v>
+      <c r="F14" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -3039,20 +3039,20 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="30" t="s">
+        <v>176</v>
+      </c>
+      <c r="C15" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="C15" s="35" t="s">
+      <c r="D15" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="E15" s="30" t="s">
         <v>178</v>
       </c>
-      <c r="D15" s="35" t="s">
-        <v>160</v>
-      </c>
-      <c r="E15" s="35" t="s">
-        <v>179</v>
-      </c>
-      <c r="F15" s="35" t="s">
-        <v>135</v>
+      <c r="F15" s="30" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -3060,20 +3060,20 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="30" t="s">
+        <v>179</v>
+      </c>
+      <c r="C16" s="30" t="s">
         <v>180</v>
       </c>
-      <c r="C16" s="35" t="s">
+      <c r="D16" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="E16" s="30" t="s">
         <v>181</v>
       </c>
-      <c r="D16" s="35" t="s">
+      <c r="F16" s="30" t="s">
         <v>134</v>
-      </c>
-      <c r="E16" s="35" t="s">
-        <v>182</v>
-      </c>
-      <c r="F16" s="35" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -3081,20 +3081,20 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="30" t="s">
+        <v>182</v>
+      </c>
+      <c r="C17" s="30" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="35" t="s">
+      <c r="D17" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="E17" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="D17" s="35" t="s">
+      <c r="F17" s="30" t="s">
         <v>134</v>
-      </c>
-      <c r="E17" s="35" t="s">
-        <v>185</v>
-      </c>
-      <c r="F17" s="35" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -3172,12 +3172,12 @@
     </row>
     <row r="3" spans="2:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="26" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" s="6">
         <f>COUNTA('1. Data Dictionary'!#REF!,'1. Data Dictionary'!#REF!)</f>
@@ -3186,7 +3186,7 @@
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C6" s="27" t="e">
         <f>SUM('1. Data Dictionary'!#REF!,'1. Data Dictionary'!#REF!)</f>
@@ -3195,7 +3195,7 @@
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" s="26" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C7" s="6">
         <f>COUNTA('1. Data Dictionary'!#REF!)+COUNTA('1. Data Dictionary'!#REF!)</f>
@@ -3204,7 +3204,7 @@
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C8" s="6">
         <f>COUNTIF('3. Data Quality Log'!F6:F20,"Open")</f>
@@ -3213,49 +3213,49 @@
     </row>
     <row r="10" spans="2:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="28" t="s">
         <v>141</v>
-      </c>
-      <c r="C10" s="28" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C11" s="28"/>
     </row>
     <row r="12" spans="2:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C12" s="28" t="s">
         <v>144</v>
-      </c>
-      <c r="C12" s="28" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" s="28" t="s">
         <v>146</v>
-      </c>
-      <c r="C13" s="28" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C14" s="28"/>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B16" s="26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C16" s="29"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C17" s="29"/>
     </row>

</xml_diff>